<commit_message>
outputs after making changes in code
</commit_message>
<xml_diff>
--- a/mcq_solving/pairwise_results_independent_style.xlsx
+++ b/mcq_solving/pairwise_results_independent_style.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:T31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,15 +548,15 @@
       <c r="G2" t="inlineStr">
         <is>
           <t>[
-  "The urogenital diaphragm is a muscular and fascial structure that spans the outlet of the pelvis.",
-  "It is composed of the deep transverse perineal muscles and the sphincter urethrae muscle, along with their associated fasciae.",
-  "Colle's fascia, also known as the subcutaneous perineal fascia, lies superficial to the urogenital diaphragm and is not a part of its structure."
+  "The urogenital diaphragm is a layer of tissue in the perineum",
+  "It consists of the deep transverse perineus muscle, the perineal body, and the sphincter urethrae muscle, as well as associated fasciae",
+  "Colles' fascia is a superficial fascia in the perineal region, not a component of the urogenital diaphragm"
 ]</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Colle's fascia is not a component of the urogenital diaphragm, which primarily consists of deep transverse perineal muscles and associated fasciae.</t>
+          <t>Colles' fascia is not part of the urogenital diaphragm</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -570,15 +570,15 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>[
-  "The urogenital diaphragm consists of the perineal membrane and the muscles and fasciae associated with it.",
-  "Colle's fascia is part of the superficial perineal pouch and lies beneath the skin and superficial perineal fascia (Scarpa's fascia).",
-  "Therefore, Colle's fascia is not a component of the urogenital diaphragm."
+  "The urogenital diaphragm is a layer of the pelvis that consists of muscle and fascia",
+  "It is primarily composed of the deep transverse perineal muscle, the perineal membrane (also known as the inferior fascia of the urogenital diaphragm), and the superior fascia of the urogenital diaphragm",
+  "Colles' fascia is a superficial layer of fascia in the perineal region, but it is not considered a component of the urogenital diaphragm itself"
 ]</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Colle's fascia is not part of the urogenital diaphragm, which includes the perineal membrane and associated structures.</t>
+          <t>Colles' fascia is not a component of the urogenital diaphragm</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -592,15 +592,15 @@
       <c r="O2" t="inlineStr">
         <is>
           <t>[
-  "The urogenital diaphragm is a structure in the pelvis that includes several layers and muscles.",
-  "Colle's fascia is part of the superficial perineal pouch and does not form part of the urogenital diaphragm.",
-  "The Sphincter Urethrae muscle is a component of the urogenital diaphragm, contributing to its function."
+  "The urogenital diaphragm is a layer of tissue in the perineum that supports the urethra and consists of two fascial layers and a muscular layer",
+  "The muscular layer is primarily composed of the sphincter urethrae, which is responsible for controlling the flow of urine",
+  "Colles' fascia is a superficial fascial layer in the perineum, but it is not a component of the urogenital diaphragm itself"
 ]</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Colle's fascia is not a component of the urogenital diaphragm, while the Sphincter Urethrae muscle is.</t>
+          <t>Colles' fascia is not a component of the urogenital diaphragm</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr"/>
@@ -642,15 +642,15 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>[
-  "Type I Diabetes can lead to diabetic retinopathy, which is a serious complication affecting the eyes.",
-  "Guidelines recommend regular screening for diabetic retinopathy to detect and treat it early.",
-  "For children with Type I Diabetes, fundus examinations should begin after 5 years of diagnosis or at puberty, whichever comes first, to ensure early detection of retinopathy."
+  "Type I Diabetes is typically diagnosed in children and adolescents",
+  "The American Academy of Pediatrics and the American Diabetes Association recommend regular screening for diabetic retinopathy",
+  "The recommended time for initial fundus examination in children with Type I Diabetes is typically after 3-5 years of disease duration, once the child is aged 10 years or older, or at puberty, whichever comes first"
 ]</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Fundus examinations should start after 5 years of diagnosis in children with Type I Diabetes to monitor for diabetic retinopathy.</t>
+          <t>Current guidelines suggest starting screening after 5 years</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -664,15 +664,15 @@
       <c r="O3" t="inlineStr">
         <is>
           <t>[
-  "Type I Diabetes can lead to diabetic retinopathy, a complication that affects the eyes.",
-  "The American Diabetes Association recommends that patients with Type I Diabetes should have an initial dilated and comprehensive eye examination within 5 years after the onset of diabetes.",
-  "This recommendation is based on the typical progression of diabetes and the risk of developing retinopathy, which generally does not occur in the first few years of diagnosis."
+  "Type I Diabetes is typically diagnosed in children and adolescents",
+  "The American Diabetes Association recommends that children with Type I Diabetes should have an initial eye examination by an ophthalmologist or optometrist experienced in diagnosing diabetic eye disease approximately 3-5 years after the onset of diabetes, once they have had diabetes for 5 years, given that the onset of Type I Diabetes often occurs at a young age and diabetic retinopathy is rare in the first 5 years of disease",
+  "Given the options, the closest recommendation aligns with having the examination after 5 years of diagnosis"
 ]</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Fundus examinations are recommended after 5 years from the time of diagnosis to monitor for diabetic retinopathy.</t>
+          <t>Recommendation aligns with standard practice for Type I Diabetes management in children</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -686,15 +686,15 @@
       <c r="S3" t="inlineStr">
         <is>
           <t>[
-  "Type I diabetes increases the risk of diabetic retinopathy, which can lead to vision loss if not detected and treated early.",
-  "Guidelines recommend that children with Type I diabetes should have their first eye examination after 5 years of diagnosis or at puberty, whichever comes first, to screen for diabetic retinopathy.",
-  "This timing allows for early detection and intervention, as retinopathy is rare before 5 years of diabetes duration in children."
+  "Type I Diabetes typically develops in children and young adults, and diabetic retinopathy is a common complication.",
+  "The American Academy of Pediatrics and the American Diabetes Association recommend regular eye exams for children with Type I Diabetes to screen for diabetic retinopathy.",
+  "The recommended time to start screening for diabetic retinopathy in children with Type I Diabetes is typically around 3-5 years after the diagnosis, or at the age of 10-11 years, whichever comes first, but for children diagnosed at age 10 or more, screening should start at the time of diagnosis."
 ]</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Children with Type I diabetes should have their first fundus examination after 5 years of diagnosis to screen for diabetic retinopathy.</t>
+          <t>Children with Type I Diabetes should have their first fundus examination approximately 3-5 years after diagnosis</t>
         </is>
       </c>
     </row>
@@ -719,24 +719,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>[
-  "The sensitivity of a test refers to its ability to correctly identify those with the disease.",
-  "The fecal antigen test has a high sensitivity, typically over 90%, and is non-invasive.",
-  "While the biopsy urease test is highly specific and useful in endoscopic settings, it is not as sensitive as the fecal antigen test."
+  "The most sensitive test for H pylori needs to be identified among the given options",
+  "Biopsy urease test, also known as rapid urease test, is highly sensitive and specific for detecting H pylori infection, especially when a biopsy sample is available",
+  "Fecal antigen test is also sensitive but the biopsy urease test is considered more sensitive due to its direct detection method from gastric mucosa"
 ]</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Fecal antigen test is more sensitive than biopsy urease test for detecting H pylori.</t>
+          <t>Biopsy urease test is more sensitive</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -745,24 +745,24 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="N4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
           <t>[
-  "The sensitivity of a diagnostic test is crucial for accurately identifying the presence of H pylori.",
-  "The biopsy urease test, while highly specific, requires an endoscopy and is invasive. It is used to confirm the presence of H pylori in tissue samples but is not the most sensitive method.",
-  "The urea breath test (UBT) is non-invasive and has high sensitivity and specificity. It detects the presence of H pylori by measuring the conversion of ingested urea into carbon dioxide, which is exhaled."
+  "The most sensitive test for H pylori needs to be identified among the given options",
+  "Biopsy urease test, also known as rapid urease test, is highly sensitive and specific for detecting H pylori",
+  "Urea breath test is also sensitive but the comparison between the two options is required to determine the most sensitive"
 ]</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>The urea breath test is the most sensitive and non-invasive test for detecting H pylori.</t>
+          <t>Biopsy urease test is considered the most sensitive</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -776,15 +776,15 @@
       <c r="S4" t="inlineStr">
         <is>
           <t>[
-  "The biopsy urease test is highly specific and sensitive for detecting active H. pylori infection in the stomach.",
-  "Serological tests can detect antibodies against H. pylori, but they cannot distinguish between past and current infections.",
-  "Given the need for sensitivity and specificity in diagnosing active infections, the biopsy urease test is superior."
+  "The most sensitive test for H pylori needs to be identified",
+  "Biopsy urease test is a direct method that detects the presence of H pylori by its urease activity, making it highly sensitive",
+  "Serological tests detect antibodies against H pylori and can be less sensitive due to potential false negatives in early infection or after treatment"
 ]</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Biopsy urease test is more sensitive and specific for detecting active H. pylori infection compared to serological tests.</t>
+          <t>Biopsy urease test is highly sensitive for H pylori detection</t>
         </is>
       </c>
     </row>
@@ -809,46 +809,46 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>[
+  "The common hepatic artery branches into the proper hepatic artery and the right gastric artery",
+  "The right gastric artery supplies the stomach, specifically the lesser curvature, and anastomoses with the left gastric artery",
+  "Ligation of the common hepatic artery would compromise blood flow to the right gastric artery, and potentially affect the left gastric artery due to their anastomosis"
+]</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Compromised blood flow to right and left gastric arteries</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="F5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>[
-  "The common hepatic artery branches into the proper hepatic artery, the gastroduodenal artery, and the right gastric artery.",
-  "The right gastric artery supplies the lesser curvature of the stomach, while the left gastric artery, which arises from the celiac trunk, also supplies the lesser curvature of the stomach.",
-  "Ligation of the common hepatic artery would affect the right gastric artery but not the left gastric artery, as the latter originates directly from the celiac trunk."
-]</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Ligation of the common hepatic artery will compromise blood flow to the right gastric and right gastroepiploic arteries, as they both originate from it.</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
       <c r="J5" t="b">
         <v>1</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>[
-  "The common hepatic artery branches into the proper hepatic artery and the gastroduodenal artery.",
-  "The gastroduodenal artery further branches into the right gastric artery and the right gastroepiploic artery.",
-  "Ligation of the common hepatic artery would therefore affect the blood supply to the right gastric and right gastroepiploic arteries."
+  "The common hepatic artery branches into the proper hepatic artery and the right gastric artery",
+  "The right gastric artery supplies the stomach, and the right gastroepiploic artery is a branch of the gastroduodenal artery, which in turn is a branch of the common hepatic artery",
+  "The short gastric arteries are branches of the splenic artery, which is not directly affected by ligation of the common hepatic artery"
 ]</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>The right gastric and right gastroepiploic arteries originate from the gastroduodenal artery, which is a branch of the common hepatic artery. Ligation of the common hepatic artery would compromise blood flow to these arteries.</t>
+          <t>Ligation of the common hepatic artery affects the right gastric and right gastroepiploic arteries</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -866,15 +866,15 @@
       <c r="S5" t="inlineStr">
         <is>
           <t>[
-  "The common hepatic artery branches into the proper hepatic artery and the gastroduodenal artery.",
-  "The gastroduodenal artery further branches into the right gastroepiploic artery and the superior pancreaticoduodenal artery.",
-  "The right gastric artery typically arises from the proper hepatic artery, while the short gastric arteries arise from the splenic artery, which is not affected by ligation of the common hepatic artery."
+  "The common hepatic artery branches into the proper hepatic artery and the right gastric artery",
+  "The right gastroepiploic artery is a branch of the gastroduodenal artery, which in turn is a branch of the common hepatic artery",
+  "The short gastric arteries typically arise from the splenic artery, not the common hepatic artery"
 ]</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Ligation of the common hepatic artery will affect the right gastric artery and the right gastroepiploic artery, as both are derived from branches of the common hepatic artery.</t>
+          <t>Ligation affects right gastric and right gastroepiploic arteries</t>
         </is>
       </c>
     </row>
@@ -912,15 +912,15 @@
       <c r="K6" t="inlineStr">
         <is>
           <t>[
-  "In the first week of typhoid fever, the bacteria Salmonella typhi are present in the bloodstream.",
-  "Blood culture is the most sensitive and specific method for detecting the presence of S. typhi in the blood during this period.",
-  "The Widal test, which detects antibodies against S. typhi, is not reliable in the first week as the body has not yet produced sufficient antibodies."
+  "In the first week of typhoid fever, the bacteria Salmonella Typhi is more likely to be present in the blood",
+  "Blood culture is the most sensitive method for detecting Salmonella Typhi in the blood during the early stages of the disease",
+  "Widal test, which detects antibodies against Salmonella Typhi, may not be positive until the second week of illness"
 ]</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Blood culture is the investigation of choice in the first week of typhoid fever due to its high sensitivity and specificity for detecting S. typhi.</t>
+          <t>Blood culture is the investigation of choice in the 1st week of typhoid</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -934,15 +934,15 @@
       <c r="O6" t="inlineStr">
         <is>
           <t>[
-  "Typhoid fever is caused by Salmonella typhi, which can be detected in blood during the first week of infection.",
-  "Blood culture is highly sensitive and specific for detecting S. typhi in the early stages of the disease.",
-  "Urine culture is less reliable for diagnosing typhoid in the first week as the bacteria are not typically present in significant amounts in urine at this stage."
+  "In the first week of typhoid fever, the bacteria Salmonella Typhi is more likely to be present in the bloodstream",
+  "Blood culture is the most sensitive method for detecting S. Typhi during this period",
+  "Urine culture may not be positive until the second week of illness, making it less suitable for early diagnosis"
 ]</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Blood culture is the investigation of choice in the first week of typhoid fever due to its high sensitivity and specificity for detecting S. typhi.</t>
+          <t>Blood culture is the investigation of choice in the 1st week of typhoid fever</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -956,15 +956,15 @@
       <c r="S6" t="inlineStr">
         <is>
           <t>[
-  "In the first week of typhoid fever, the bacteria are present in the bloodstream.",
-  "Blood culture has a higher sensitivity for detecting Salmonella typhi in the first week of illness compared to stool culture.",
-  "Stool culture becomes more useful in the second and third weeks of the disease."
+  "In the first week of typhoid fever, the bacteria Salmonella Typhi is more likely to be present in the bloodstream",
+  "Blood culture is the most sensitive method for detecting S. Typhi during this period",
+  "Stool culture may not be positive until the second or third week of illness, making it less useful for early diagnosis"
 ]</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Blood culture is the investigation of choice in the first week of typhoid fever due to higher sensitivity for detecting Salmonella typhi in the bloodstream.</t>
+          <t>Blood culture is the investigation of choice in the 1st week of typhoid</t>
         </is>
       </c>
     </row>
@@ -998,15 +998,15 @@
       <c r="G7" t="inlineStr">
         <is>
           <t>[
-  "Sulphuric acid and nitric acid are both strong acids that can cause significant tissue damage upon contact.",
-  "Sulphuric acid is more viscous and tends to coagulate proteins, leading to a protective layer that may limit deeper penetration.",
-  "Nitric acid is less viscous and can penetrate tissues more deeply, causing more extensive damage and increasing the risk of perforation."
+  "Perforation of the stomach due to acid ingestion is a serious condition",
+  "Sulphuric acid and nitric acid are both corrosive substances, but their effects on the stomach lining differ",
+  "Nitric acid is more likely to cause perforation due to its strong oxidizing properties and ability to penetrate tissues"
 ]</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Nitric acid is more likely to cause perforation due to its ability to penetrate tissues more deeply.</t>
+          <t>Nitric acid's oxidizing properties increase risk of perforation</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -1024,15 +1024,15 @@
       <c r="O7" t="inlineStr">
         <is>
           <t>[
-  "Sulphuric acid (Option B) is a strong acid that can cause severe chemical burns and tissue necrosis upon contact with the gastrointestinal mucosa.",
-  "Carbolic acid (Option D), also known as phenol, is highly toxic and corrosive but is less likely to cause immediate physical perforation compared to sulphuric acid.",
-  "Given the corrosive nature and the immediate tissue damage potential, sulphuric acid is more likely to cause perforation of the stomach."
+  "Perforation of the stomach due to ingestion of a substance is more likely to occur with highly corrosive agents",
+  "Sulphuric acid is a highly corrosive strong mineral acid that can cause severe burns upon contact with tissues, including the stomach lining",
+  "Carbolic acid, while toxic, is less corrosive compared to sulphuric acid and more likely to cause systemic toxicity rather than immediate perforation"
 ]</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Sulphuric acid is more likely to cause immediate and severe damage leading to perforation due to its strong corrosive properties.</t>
+          <t>Sulphuric acid is more corrosive</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1046,15 +1046,15 @@
       <c r="S7" t="inlineStr">
         <is>
           <t>[
-  "Sulphuric acid (H2SO4) and hydrochloric acid (HCl) are both strong acids, but they have different properties that affect their corrosive potential.",
-  "Sulphuric acid is more dehydrating and can cause more severe tissue damage due to its ability to remove water from tissues, leading to coagulative necrosis.",
-  "Hydrochloric acid, while also corrosive, is less likely to cause perforation compared to sulphuric acid because it does not dehydrate tissues as aggressively."
+  "Perforation of the stomach due to ingestion of a substance is more likely to occur with a highly corrosive agent",
+  "Sulphuric acid is a highly corrosive strong mineral acid with dehydrating properties, capable of causing severe burns upon contact with tissues",
+  "Hydrochloric acid, while also corrosive, is naturally produced in the stomach and thus the stomach lining has some natural defense against it, making sulphuric acid more likely to cause perforation"
 ]</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Sulphuric acid is more likely to cause perforation due to its stronger dehydrating properties and greater tissue damage potential.</t>
+          <t>Sulphuric acid is more corrosive</t>
         </is>
       </c>
     </row>
@@ -1092,15 +1092,15 @@
       <c r="K8" t="inlineStr">
         <is>
           <t>[
-  "Brown tumors are benign bone lesions that occur in hyperparathyroidism.",
-  "They result from increased osteoclastic activity due to high levels of parathyroid hormone (PTH).",
-  "Hypoparathyroidism does not cause brown tumors as it is characterized by low PTH levels."
+  "Brown tumour is a bone lesion that occurs due to increased osteoclastic activity",
+  "This increased osteoclastic activity is typically seen in conditions with elevated parathyroid hormone levels",
+  "Hyperparathyroidism is characterized by an overproduction of parathyroid hormone, which can lead to the development of brown tumours"
 ]</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Brown tumors are associated with hyperparathyroidism due to increased osteoclastic activity.</t>
+          <t>Hyperparathyroidism causes increased parathyroid hormone levels leading to brown tumour formation</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1114,15 +1114,15 @@
       <c r="O8" t="inlineStr">
         <is>
           <t>[
-  "Brown tumors are associated with conditions that cause prolonged elevation of parathyroid hormone (PTH).",
-  "Hyperparathyroidism is characterized by excessive production of PTH, which can lead to bone resorption and the formation of brown tumors.",
-  "Hyperthyroidism involves overactivity of the thyroid gland and does not directly cause the formation of brown tumors."
+  "Brown tumour is a bone lesion",
+  "It is characterized by an abnormal proliferation of osteoclasts and fibrous tissue",
+  "This condition is associated with hyperparathyroidism, which leads to an overproduction of parathyroid hormone, causing bone resorption"
 ]</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Brown tumors are a manifestation of hyperparathyroidism due to increased PTH levels leading to bone resorption.</t>
+          <t>Hyperparathyroidism causes brown tumour</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1136,15 +1136,2085 @@
       <c r="S8" t="inlineStr">
         <is>
           <t>[
-  "Brown tumors are associated with primary or secondary hyperparathyroidism.",
-  "They result from the excessive activity of osteoclasts due to high levels of parathyroid hormone (PTH).",
-  "Hypothyroidism does not lead to the formation of brown tumors."
+  "Brown tumour is a bone lesion",
+  "It is associated with increased osteoclastic activity",
+  "Hyperparathyroidism leads to increased osteoclastic activity due to elevated parathyroid hormone levels"
 ]</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Brown tumors are a manifestation of hyperparathyroidism, not hypothyroidism.</t>
+          <t>Hyperparathyroidism causes brown tumour</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7144</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>The technique for accurate quantification of gene expression is</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Real-Time Reverse Transcriptase PCR</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>[
+  "Real-Time Reverse Transcriptase PCR is a sensitive and quantitative method for detecting and quantifying gene expression",
+  "Northern blot is a technique used for detecting RNA, but it is not as quantitative as Real-Time Reverse Transcriptase PCR",
+  "Real-Time Reverse Transcriptase PCR provides accurate and reliable results for gene expression quantification"
+]</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Real-Time Reverse Transcriptase PCR is more quantitative</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>[
+  "Identify the purpose of the question, which is to determine the technique for accurate quantification of gene expression",
+  "Recognize that Real-Time Reverse Transcriptase PCR is a specific type of PCR that is designed for quantitative analysis of gene expression",
+  "Eliminate Option B as it is a broader category that includes many types of PCR, not all of which are suitable for quantitative analysis"
+]</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Real-Time Reverse Transcriptase PCR is specifically designed for quantitative analysis of gene expression</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="N9" t="b">
+        <v>1</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>[
+  "Gene expression quantification requires precise measurement of mRNA levels",
+  "Real-Time Reverse Transcriptase PCR (RT-PCR) is a technique that allows for the quantitative measurement of mRNA levels in real-time",
+  "Reverse Transcriptase PCR without real-time capability does not provide quantitative measurement of gene expression"
+]</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Real-Time Reverse Transcriptase PCR is the gold standard for quantitative gene expression analysis</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>7145</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>A patient presents to the doctor with diplopia when looking towards the right. On examination, he is unable to move his right eye laterally past the midline. Damage to which of these nerves would produce this clinical presentation?</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Abducent nerve</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>[
+  "The patient presents with diplopia when looking towards the right, indicating a problem with eye movement.",
+  "The inability to move the right eye laterally past the midline suggests a problem with abduction, which is the movement of the eye away from the midline of the face.",
+  "The abducent nerve (cranial nerve VI) is responsible for controlling the lateral rectus muscle, which is the primary muscle involved in abduction of the eye."
+]</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>The abducent nerve controls lateral eye movement</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N10" t="b">
+        <v>1</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>[
+  "The patient presents with diplopia when looking towards the right, indicating a problem with eye movement.",
+  "The inability to move the right eye laterally past the midline suggests a problem with abduction, which is the movement of the eye away from the midline of the face.",
+  "The abducent nerve (cranial nerve VI) is responsible for controlling the lateral rectus muscle, which is the primary muscle involved in abduction of the eye."
+]</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Damage to the abducent nerve would result in inability to abduct the eye</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="R10" t="b">
+        <v>1</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>[
+  "The patient presents with diplopia when looking towards the right, indicating a problem with eye movement.",
+  "The inability to move the right eye laterally past the midline suggests a problem with abduction, which is controlled by the lateral rectus muscle.",
+  "The lateral rectus muscle is innervated by the abducent nerve, so damage to this nerve would produce the described clinical presentation."
+]</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Damage to the abducent nerve affects lateral rectus muscle function, causing inability to abduct the eye.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>7148</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>The arrow marked structure is which part of corpus callosum:</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Splenium</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>[
+  "The corpus callosum is a thick bundle of nerve fibers that connects the two cerebral hemispheres",
+  "It has four parts: rostrum, genu, body, and splenium",
+  "The splenium is the posterior part of the corpus callosum, which matches the description of the arrow marked structure"
+]</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Splenium is the posterior part of corpus callosum</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J11" t="b">
+        <v>1</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>[
+  "The corpus callosum is a thick bundle of nerve fibers that connects the two hemispheres of the brain.",
+  "It has four main parts: the rostrum, genu, body, and splenium.",
+  "The splenium is the posterior part of the corpus callosum, which matches the location of the arrow marked structure."
+]</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>The arrow marked structure is located at the posterior part of the corpus callosum, which is the splenium.</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="R11" t="b">
+        <v>1</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>[
+  "The corpus callosum is a thick bundle of nerve fibers that connects the two hemispheres of the brain.",
+  "It has several parts, including the rostrum, genu, body, and splenium.",
+  "The splenium is the posterior part of the corpus callosum, which is typically thicker and more rounded."
+]</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>The splenium is the posterior part of the corpus callosum</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>7149</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Cytosolic cytochrome C plays an impoant function in -</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Apoptosis</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J12" t="b">
+        <v>1</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>[
+  "Cytosolic cytochrome C is a key protein involved in the intrinsic pathway of apoptosis",
+  "During apoptosis, cytochrome C is released from the mitochondria into the cytosol, where it binds to Apaf-1 and forms the apoptosome",
+  "The formation of the apoptosome triggers a cascade of reactions leading to the activation of caspases and ultimately cell death"
+]</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Cytosolic cytochrome C is a crucial component of the apoptotic pathway</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N12" t="b">
+        <v>1</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>[
+  "Cytosolic cytochrome C is a key protein involved in various cellular processes",
+  "Apoptosis, or programmed cell death, is a process where cytochrome C plays a crucial role by triggering the caspase cascade",
+  "Cell division, on the other hand, is a process that involves the replication and separation of cellular components, but cytochrome C is not directly involved in this process"
+]</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Cytosolic cytochrome C triggers apoptosis</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="R12" t="b">
+        <v>1</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>[
+  "Cytosolic cytochrome C is involved in initiating apoptosis when released from the mitochondria",
+  "Apoptosis is a process of programmed cell death, and cytochrome C plays a crucial role in this process by activating caspases",
+  "In contrast, the electron transport chain is a process that occurs in the mitochondrial inner membrane, where cytochrome C is normally located, but the question specifically asks about cytosolic cytochrome C"
+]</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Cytosolic cytochrome C initiates apoptosis</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>7150</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Trigeminal nerve has how many nucleus?</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>[
+  "The trigeminal nerve is a complex nerve with multiple functions, including sensory and motor functions.",
+  "It has several nuclei in the brainstem that are responsible for these functions, including the main sensory nucleus, spinal trigeminal nucleus, motor nucleus, and mesencephalic nucleus.",
+  "Considering the main functions and the anatomy of the trigeminal nerve, it is known to have four distinct nuclei."
+]</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Trigeminal nerve has 4 nuclei</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J13" t="b">
+        <v>1</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>[
+  "The trigeminal nerve is a complex nerve with multiple functions, including sensory and motor functions.",
+  "It has several nuclei in the brainstem that are responsible for these functions, including the main sensory nucleus, the spinal trigeminal nucleus, and the motor nucleus.",
+  "In addition to these, there is also the mesencephalic nucleus, which is involved in proprioception."
+]</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>The trigeminal nerve has 4 nuclei.</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="N13" t="b">
+        <v>1</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>[
+  "The trigeminal nerve is a complex nerve with multiple functions, including sensory and motor functions.",
+  "It has several nuclei in the brainstem that are responsible for these functions, including the main sensory nucleus, spinal trigeminal nucleus, and motor nucleus.",
+  "The correct number of nuclei for the trigeminal nerve is 4: the main sensory nucleus, spinal trigeminal nucleus, mesencephalic nucleus, and motor nucleus."
+]</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>The trigeminal nerve has 4 nuclei.</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>7151</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>The deformity of tibia in triple deformity of the knee is?</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Flexion, posterior subluxation &amp; external rotation</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>[
+  "The triple deformity of the knee is characterized by a combination of flexion, posterior subluxation, and external rotation.",
+  "This deformity typically results from a severe injury or condition affecting the knee joint, such as a fracture or neurological disorder.",
+  "Given the characteristics of the triple deformity, the correct description must include flexion, not extension, as the deformity involves a bending of the knee."
+]</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Flexion is a key component of the triple deformity</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N14" t="b">
+        <v>1</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>[
+  "Identify the components of triple deformity of the knee",
+  "Recognize that triple deformity involves flexion, posterior subluxation, and external rotation",
+  "Apply knowledge of orthopedic deformities to select the correct option"
+]</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Triple deformity of the knee is characterized by flexion, posterior subluxation, and external rotation</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="R14" t="b">
+        <v>1</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>[
+  "The triple deformity of the knee is characterized by a combination of flexion, posterior subluxation, and rotation of the tibia.",
+  "In this deformity, the tibia is typically externally rotated in relation to the femur.",
+  "This is because the posterior subluxation of the tibia tends to cause an external rotation due to the anatomy of the knee joint and the direction of the dislocation."
+]</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>External rotation is a component of the triple deformity of the knee</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>7154</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>What is the most common site of origin of thrombotic pulmonary emboli?</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Deep leg veins</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J15" t="b">
+        <v>1</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>[
+  "Thrombotic pulmonary emboli typically arise from venous thrombi that break loose and travel to the lungs",
+  "The most common source of these venous thrombi is the deep veins of the lower extremities, due to conditions such as deep vein thrombosis (DVT)",
+  "The lumen of the left ventricle is not a typical source of thrombotic pulmonary emboli, as these emboli originate from the venous system, not the arterial system"
+]</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Deep leg veins are the most common site of origin of thrombotic pulmonary emboli due to DVT</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N15" t="b">
+        <v>1</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>[
+  "Thrombotic pulmonary emboli typically arise from venous thrombi that break loose and travel to the lungs",
+  "The most common sites for venous thrombi formation are the deep veins of the lower extremities, due to factors like stasis, hypercoagulability, and endothelial injury",
+  "The deep leg veins, particularly those in the calf and thigh, are prone to thrombosis due to their dependence on muscle contraction for blood flow and the higher pressure within these veins"
+]</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Deep leg veins are the most common source of pulmonary emboli</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="R15" t="b">
+        <v>1</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>[
+  "Thrombotic pulmonary emboli typically arise from venous thrombi that break loose and travel to the lungs",
+  "The most common sites for venous thrombi formation are the deep veins of the lower extremities, particularly the iliofemoral veins",
+  "The lumen of the right ventricle is not a typical site for thrombus formation that leads to pulmonary embolism"
+]</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Deep leg veins are the most common source of thrombi that cause pulmonary embolism</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>7156</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Which of the following nipple discharge is most probably; physiological:</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>B/L milky discharge with squeezing from multiple ducts</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F16" t="b">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>[
+  "Physiological nipple discharge is typically bilateral and can be induced by squeezing the nipple",
+  "Milky discharge is a common characteristic of physiological nipple discharge, especially when it occurs in multiple ducts",
+  "Spontaneous discharge, on the other hand, can be a sign of an underlying pathological condition"
+]</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Bilateral milky discharge with squeezing from multiple ducts is more indicative of physiological nipple discharge</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N16" t="b">
+        <v>1</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>[
+  "Physiological nipple discharge is typically bilateral and milky in nature",
+  "It often involves multiple ducts and can be expressed with squeezing",
+  "Bloody discharge, especially from a single duct, is more concerning for pathological causes such as ductal carcinoma"
+]</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Bilateral milky discharge from multiple ducts is characteristic of physiological galactorrhea</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="R16" t="b">
+        <v>1</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>[
+  "Physiological nipple discharge is typically bilateral and milky in nature",
+  "It often occurs when the nipple is squeezed and can come from multiple ducts",
+  "Bloody discharge, especially unilateral, is more concerning for a pathological cause such as a breast tumor or ductal ectasia"
+]</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Bilateral milky discharge is consistent with physiological galactorrhea</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>7157</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Hallmark of breast malignancy on mammography?</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Clusters of microcalcification</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F17" t="b">
+        <v>1</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>[
+  "Breast malignancy on mammography is often characterized by specific features",
+  "Clusters of microcalcification are a known indicator of breast cancer, particularly in cases of ductal carcinoma in situ",
+  "Low density lesions are not typically a hallmark of malignancy, as malignant lesions are often of higher density than the surrounding breast tissue"
+]</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Clusters of microcalcification are a classic sign of breast malignancy</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J17" t="b">
+        <v>1</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>[
+  "Breast malignancy on mammography is often characterized by specific features",
+  "Clusters of microcalcification are a known indicator of breast cancer, particularly in cases of ductal carcinoma in situ",
+  "Smooth margins are more commonly associated with benign lesions"
+]</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Microcalcification clusters are a hallmark of malignancy</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="N17" t="b">
+        <v>1</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>[
+  "Breast malignancy on mammography is often characterized by specific patterns of calcification",
+  "Clusters of microcalcification are typically associated with malignant breast lesions, as they can represent ductal carcinoma in situ or invasive cancer",
+  "Popcorn calcification is more commonly seen in benign lesions, such as fibroadenomas"
+]</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Clusters of microcalcification are a hallmark of breast malignancy</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>7159</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Computed Tomography (CT scan) is least accurate for diagnosts of:</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1cm size Gall stones</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F18" t="b">
+        <v>1</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>[
+  "CT scans are highly sensitive for detecting vascular abnormalities, such as aneurysms, due to the use of contrast agents that highlight blood vessels",
+  "Gallstones, especially those larger than 1cm, are typically visible on CT scans due to their density difference from surrounding tissues",
+  "However, small gallstones or those with similar density to bile may be missed, but the accuracy for 1cm size gallstones is generally high"
+]</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>CT scans are less accurate for small or isodense gallstones</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J18" t="b">
+        <v>0</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>[
+  "CT scans are highly sensitive for detecting gallstones, especially those larger than 1cm in size",
+  "The density of gallstones, particularly those composed of calcium, makes them easily visible on CT scans",
+  "In contrast, small lymph nodes, even those larger than 1cm, can be more challenging to accurately assess on CT scans due to their size, location, and potential for partial volume averaging"
+]</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>CT scans are less accurate for diagnosing small lymph nodes</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="R18" t="b">
+        <v>0</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>[
+  "CT scans are highly sensitive for detecting gallstones, especially those larger than 1cm in size due to their high density",
+  "The tail of the pancreas is a challenging area to visualize due to its location and the presence of surrounding structures, making CT scans less accurate for detecting small masses",
+  "Given the size of 1cm, a mass in the tail of the pancreas would be more difficult to accurately diagnose with a CT scan compared to a 1cm gallstone"
+]</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>CT scans are less accurate for small pancreatic masses due to location and surrounding structures</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>7161</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>NO is synthesized by -</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Arginine</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F19" t="b">
+        <v>1</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>[
+  "Nitric oxide (NO) is a crucial signaling molecule in the body",
+  "The synthesis of NO involves the enzyme nitric oxide synthase (NOS), which catalyzes the conversion of the amino acid L-arginine to citrulline, producing NO as a byproduct",
+  "Uracil is a nucleotide base found in RNA, not directly involved in NO synthesis"
+]</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Arginine is the direct precursor to NO synthesis</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J19" t="b">
+        <v>1</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>[
+  "Nitric oxide (NO) synthesis involves the conversion of a specific amino acid",
+  "The enzyme responsible for this conversion is nitric oxide synthase (NOS)",
+  "NOS catalyzes the conversion of L-arginine to L-citrulline, producing NO as a byproduct"
+]</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Arginine is the precursor for NO synthesis</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="R19" t="b">
+        <v>1</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>[
+  "Nitric oxide (NO) is a crucial signaling molecule in the body",
+  "The synthesis of NO is primarily catalyzed by the enzyme nitric oxide synthase (NOS)",
+  "NOS uses the amino acid L-arginine as its substrate to produce NO and citrulline"
+]</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Arginine is the direct precursor for NO synthesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>7162</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>The serum concentration of which of the following human Ig is maximum:</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>IgG</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J20" t="b">
+        <v>1</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>[
+  "IgG is the most abundant antibody isotype in human serum",
+  "It constitutes approximately 75-80% of the total serum immunoglobulins",
+  "IgG provides the majority of antibody-based immunity against invading pathogens"
+]</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>IgG is the most abundant antibody in human serum</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N20" t="b">
+        <v>1</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>[
+  "IgG is the most abundant antibody isotype in the human serum",
+  "It provides the majority of antibody-based immunity against invading pathogens",
+  "IgD is primarily found on the surface of mature B cells, not in high concentrations in serum"
+]</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>IgG is the most abundant antibody in human serum</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="R20" t="b">
+        <v>1</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>[
+  "Identify the types of human immunoglobulins (Ig) and their typical serum concentrations",
+  "Recall that IgG is the most abundant, making up about 75-80% of the total serum immunoglobulins",
+  "Compare this with IgM, which is the first antibody to be made by the body to fight a new infection but is present in lower concentrations than IgG"
+]</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>IgG is the most abundant immunoglobulin in human serum</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>7166</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Arlts line is seen in</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Trachoma</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F21" t="b">
+        <v>1</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>[
+  "Arlts line is a characteristic feature of trachoma, which is a chronic keratoconjunctivitis caused by Chlamydia trachomatis",
+  "Trachoma is known to cause scarring of the tarsal conjunctiva, leading to the formation of Arlts line",
+  "Vernal keratoconjunctivitis is a seasonal allergic disorder, and it does not typically cause the formation of Arlts line"
+]</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Arlts line is a specific sign of trachoma</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J21" t="b">
+        <v>1</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>[
+  "Arlts line is a characteristic feature of a specific eye condition",
+  "Trachoma is a chronic keratoconjunctivitis caused by Chlamydia trachomatis, which can lead to the formation of Arlt's line",
+  "Pterygium is a growth of the conjunctiva or mucous membrane that covers the white part of the eye, but it is not typically associated with Arlt's line"
+]</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Arlts line is a characteristic feature of Trachoma</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="R21" t="b">
+        <v>1</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>[
+  "Arlts line is a characteristic sign of trachoma, which is a chronic keratoconjunctivitis caused by Chlamydia trachomatis",
+  "Trachoma is known to cause scarring of the tarsal conjunctiva, leading to the formation of Arlt's line",
+  "Ocular pemphigoid, on the other hand, is an autoimmune disease that primarily affects the conjunctiva and cornea, but it is not typically associated with Arlt's line"
+]</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Arlts line is a specific sign of trachoma</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>7168</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>A young male patient presents with complete rectal prolapse. The surgery of choice is</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Abdominal rectopexy</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J22" t="b">
+        <v>1</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>[
+  "Identify the condition as complete rectal prolapse, which requires a surgical intervention to restore the normal position of the rectum",
+  "Consider the surgical options for rectal prolapse, including abdominal rectopexy and Delerom's procedure (also known as Delorme's procedure)",
+  "Abdominal rectopexy is generally considered the surgery of choice for younger patients with complete rectal prolapse due to its effectiveness in correcting the prolapse and minimizing recurrence, whereas Delorme's procedure is often reserved for older or higher-risk patients"
+]</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Abdominal rectopexy is the preferred surgical approach for a young male patient with complete rectal prolapse</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N22" t="b">
+        <v>1</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>[
+  "Complete rectal prolapse is a condition where the rectum loses its normal attachments and protrudes out of the anus",
+  "Abdominal rectopexy is a surgical procedure that involves fixing the rectum to the sacrum to correct rectal prolapse",
+  "Goodsall's procedure is related to the treatment of anal fistulas, not rectal prolapse"
+]</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Abdominal rectopexy is the standard surgical treatment for complete rectal prolapse</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="R22" t="b">
+        <v>1</v>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>[
+  "Complete rectal prolapse is a condition where the rectum loses its normal attachments inside the body, allowing it to protrude out through the anus",
+  "Abdominal rectopexy is a surgical procedure that involves attaching the rectum to the sacrum with mesh to prevent further prolapse, addressing the root cause of the condition",
+  "Anterior resection is typically used to treat rectal cancer or other conditions affecting the rectum, not specifically for rectal prolapse"
+]</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Abdominal rectopexy directly addresses the issue of rectal prolapse</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>7169</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>The drug that inhibits uterine contractility and cause pulmonary edema is:</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ritodrine</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J23" t="b">
+        <v>1</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>[
+  "Ritodrine is a beta-2 adrenergic agonist used to inhibit uterine contractility",
+  "Ritodrine can cause pulmonary edema as a side effect due to its beta-2 agonist activity leading to fluid retention",
+  "Nifedipine is a calcium channel blocker also used to inhibit uterine contractility but it is less commonly associated with pulmonary edema compared to ritodrine"
+]</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Ritodrine is known for causing pulmonary edema</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N23" t="b">
+        <v>1</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>[
+  "Ritodrine is a beta-2 adrenergic agonist used to inhibit uterine contractility",
+  "Ritodrine can cause pulmonary edema as a side effect due to its beta-2 agonist activity leading to fluid retention and potential heart rate increases",
+  "Atosiban is an oxytocin/vasopressin receptor antagonist that also inhibits uterine contractility but is not commonly associated with causing pulmonary edema"
+]</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Ritodrine causes pulmonary edema</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="R23" t="b">
+        <v>1</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>[
+  "Ritodrine is a beta-2 adrenergic agonist used to inhibit uterine contractions",
+  "Ritodrine can cause fluid retention and pulmonary edema as a side effect",
+  "Indomethacin is a nonsteroidal anti-inflammatory drug (NSAID) that can actually reduce uterine contractions but is not typically associated with causing pulmonary edema"
+]</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Ritodrine inhibits uterine contractility and can cause pulmonary edema</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>7170</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Influenzae virus belongs to which family?</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Orthomyxovirus</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F24" t="b">
+        <v>1</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>[
+  "Influenza virus classification is based on its genetic and antigenic properties",
+  "Orthomyxovirus family includes influenza viruses, which are known for their segmented RNA genome",
+  "Paramyxovirus family includes different viruses such as measles and mumps, not influenza"
+]</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Influenza virus is classified under Orthomyxovirus family</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N24" t="b">
+        <v>1</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>[
+  "Influenza virus classification is based on its genetic and antigenic properties",
+  "Orthomyxovirus family includes viruses with segmented single-stranded RNA genomes, which matches the characteristics of Influenza virus",
+  "Togaviridae family includes viruses with positive-sense single-stranded RNA genomes, which does not match the characteristics of Influenza virus"
+]</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Influenza virus is a type of Orthomyxovirus</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="R24" t="b">
+        <v>1</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>[
+  "Identify the virus in question: Influenzae virus",
+  "Recall the classification of Influenzae virus: it is a type of RNA virus",
+  "Determine the correct family for Influenzae virus: Orthomyxovirus is the correct family"
+]</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Influenzae virus belongs to the Orthomyxovirus family</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>7173</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Several weeks after surgical dissection of her left axilla for the removal of lymph nodes for staging and treatment of her breast cancer, a 32-year-old woman was told by her general physician that she had "winging" of her left scapula when she pushed against resistance during her physical examination. She told the physician that she had also experienced difficulty lately in raising her right arm above her head when she was combing her hair. In a subsequent consult visit with her surgeon, she was told that a nerve was accidentally injured during the diagnostic surgical procedure and that this produced her scapular abnormality and inability to raise her arm normally. What was the origin of this nerve?</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Roots of the brachial plexus</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F25" t="b">
+        <v>1</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>[
+  "The patient presents with winging of the left scapula, which is typically associated with weakness of the serratus anterior muscle, supplied by the long thoracic nerve.",
+  "However, the long thoracic nerve originates from the roots of the brachial plexus, specifically C5-C7.",
+  "The patient also experiences difficulty raising her right arm above her head, which suggests a problem with the right arm, not directly related to the left axilla surgery, but the question focuses on the nerve injury causing the scapular abnormality on the left side."
+]</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>The long thoracic nerve, which causes winging of the scapula when damaged, originates from the roots of the brachial plexus.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J25" t="b">
+        <v>1</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>[
+  "The patient presents with winging of the left scapula, which is typically associated with weakness of the serratus anterior muscle, supplied by the long thoracic nerve.",
+  "The long thoracic nerve originates from the roots of the brachial plexus, specifically from the C5, C6, and sometimes C7 roots.",
+  "Difficulty in raising the right arm above the head is not directly related to the described symptoms on the left side, suggesting either an unrelated issue or a mistake in the question's details, but the focus remains on the nerve responsible for the scapular winging on the left side."
+]</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>The long thoracic nerve, which causes scapular winging when damaged, originates from the roots of the brachial plexus.</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="N25" t="b">
+        <v>1</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>[
+  "The patient presents with winging of the left scapula, which is typically associated with weakness of the serratus anterior muscle, supplied by the long thoracic nerve.",
+  "However, the long thoracic nerve originates from the roots of the brachial plexus, specifically from the C5, C6, and sometimes C7 roots.",
+  "The difficulty in raising the right arm above her head could be a red herring, but the specific symptom of scapular winging points towards an injury to a nerve originating from the roots of the brachial plexus."
+]</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>The long thoracic nerve originates from the roots of the brachial plexus.</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>7174</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Post transplant lymphoma is ?</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>B cell</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F26" t="b">
+        <v>1</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>[
+  "Post-transplant lymphoproliferative disorders (PTLD) are a well-recognized complication of solid organ transplantation and bone marrow transplantation",
+  "The majority of PTLD cases are of B-cell origin, often associated with Epstein-Barr virus (EBV) infection",
+  "Given the context, the most accurate answer regarding post-transplant lymphoma would be related to B cells, not T cells"
+]</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>B cell lymphomas are more common in post-transplant patients</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N26" t="b">
+        <v>1</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>[
+  "Post-transplant lymphoproliferative disorders (PTLD) are a well-recognized complication of solid organ transplantation and bone marrow transplantation",
+  "The majority of PTLD cases are of B-cell origin, often associated with Epstein-Barr virus (EBV) infection",
+  "NK cell lymphomas are rare and not typically associated with post-transplant lymphoproliferative disorders"
+]</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>B cell lymphomas are the most common type of post-transplant lymphoma</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="R26" t="b">
+        <v>1</v>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>[
+  "Post-transplant lymphoproliferative disorders (PTLD) are a well-recognized complication of solid organ transplantation and bone marrow transplantation",
+  "The majority of PTLD cases are of B-cell origin, often associated with Epstein-Barr virus (EBV) infection",
+  "B cells are the primary cell type involved in the development of post-transplant lymphomas"
+]</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>B cell lymphomas are the most common type of post-transplant lymphoma</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>7175</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>The following insulin can be given intravenously?</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Regular insulin</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F27" t="b">
+        <v>1</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>[
+  "Regular insulin is a short-acting insulin that can be administered intravenously due to its rapid onset of action",
+  "Protamine zinc insulin is an intermediate-acting insulin with a slower onset of action, typically given subcutaneously",
+  "Intravenous administration requires rapid action, making Regular insulin the suitable choice"
+]</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Regular insulin can be given intravenously due to its pharmacokinetic properties</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J27" t="b">
+        <v>1</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>[
+  "Regular insulin has a fast onset of action and can be administered intravenously for rapid glucose control",
+  "Ultra lente insulin has a slow onset and long duration of action, making it less suitable for intravenous administration",
+  "Intravenous administration of insulin requires a rapid-acting form to achieve immediate effects"
+]</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Regular insulin is suitable for intravenous use</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="R27" t="b">
+        <v>1</v>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>[
+  "Regular insulin is a short-acting insulin that can be administered intravenously due to its quick onset of action and short duration",
+  "Semi lente insulin is an intermediate-acting insulin that is not suitable for intravenous administration due to its slower onset and longer duration",
+  "Intravenous administration of insulin requires a rapid onset of action, which is characteristic of regular insulin"
+]</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Regular insulin is suitable for intravenous administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>7177</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Megaloblastic anemia, glossitis, pharyngeal ulcers, and impaired immunity. For each disorder above, select the dietary deficiency that is likely to be responsible.</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Folate deficiency</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J28" t="b">
+        <v>1</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>[
+  "Megaloblastic anemia is typically associated with deficiencies in either vitamin B12 or folate, as both are crucial for DNA synthesis and red blood cell production.",
+  "Glossitis and pharyngeal ulcers can also be symptoms of folate deficiency, among other conditions, due to the role of folate in maintaining mucosal health.",
+  "Impaired immunity can result from various nutritional deficiencies, but given the combination with megaloblastic anemia, folate deficiency is a more direct link than thiamine deficiency."
+]</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Folate deficiency matches the symptoms described.</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N28" t="b">
+        <v>1</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>[
+  "Megaloblastic anemia is typically associated with deficiencies in either vitamin B12 or folate, as both are crucial for DNA synthesis and red blood cell production.",
+  "Glossitis and pharyngeal ulcers can also be symptoms of folate deficiency, as folate is important for the health of the mucous membranes and the gastrointestinal system.",
+  "Impaired immunity can be linked to folate deficiency as well, since folate plays a role in the functioning of the immune system."
+]</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Folate deficiency matches all symptoms described</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="R28" t="b">
+        <v>1</v>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>[
+  "Megaloblastic anemia is typically associated with deficiencies in either vitamin B12 or folate",
+  "Glossitis and pharyngeal ulcers can also be related to folate deficiency, among other causes",
+  "Impaired immunity can be linked to folate deficiency due to its role in DNA synthesis and repair, which is crucial for immune cell function"
+]</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Folate deficiency matches all described conditions</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>7178</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Tamsulosin belongs to</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>a1a receptor blockers</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F29" t="b">
+        <v>1</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>[
+  "Identify the drug Tamsulosin",
+  "Determine the class of the drug",
+  "Recognize that Tamsulosin is primarily used to treat benign prostatic hyperplasia by relaxing the muscles in the prostate and bladder neck, making it an alpha-1 adrenergic receptor blocker"
+]</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Tamsulosin is an alpha-1a receptor blocker</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N29" t="b">
+        <v>1</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>[
+  "Tamsulosin is a medication used to treat benign prostatic hyperplasia (BPH) and other conditions",
+  "It works by relaxing the muscles in the prostate and bladder neck, making it easier to urinate",
+  "Tamsulosin is classified as an alpha-1 adrenergic receptor blocker, which is a type of medication that blocks the action of alpha-1 adrenergic receptors in the smooth muscle of the prostate and bladder neck"
+]</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Tamsulosin is an alpha-1a receptor blocker</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="R29" t="b">
+        <v>1</v>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>[
+  "Tamsulosin is a medication used to treat benign prostatic hyperplasia (BPH)",
+  "It works by relaxing the muscles in the prostate and bladder neck, making it easier to urinate",
+  "Tamsulosin is classified as an alpha-1 adrenergic receptor blocker, specifically an alpha-1a receptor blocker"
+]</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Tamsulosin is an alpha-1a receptor blocker</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>7181</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>A patient with H. Pylori infection is treated with drugs. The best method to detect presence of residual H.Pylori infection in this person is which of the following?</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Urea breath test</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F30" t="b">
+        <v>1</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>[
+  "The patient has been treated with drugs, so a test that directly detects the bacteria or its components may not be reliable due to potential false negatives.",
+  "The urea breath test detects the presence of active H. Pylori infection by measuring the amount of carbon dioxide produced when the bacteria break down urea.",
+  "The rapid urease test requires a sample of gastric mucosa, which may not be feasible or accurate after treatment, whereas the urea breath test is non-invasive and can be performed after treatment."
+]</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Urea breath test is more accurate for detecting residual H. Pylori infection after treatment.</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N30" t="b">
+        <v>1</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>[
+  "H. Pylori infection is a bacterial infection that can be treated with antibiotics",
+  "The urea breath test detects the presence of active H. Pylori bacteria by measuring the amount of carbon dioxide produced when the bacteria break down urea",
+  "Serum anti H.Pylori titre measures the level of antibodies against H. Pylori, which can remain elevated even after successful treatment"
+]</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Urea breath test is more accurate for detecting active H. Pylori infection</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="R30" t="b">
+        <v>1</v>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>[
+  "H. Pylori infection is a bacterial infection that can be treated with antibiotics, but verification of eradication is necessary to ensure the infection is fully cleared",
+  "The urea breath test is a non-invasive and highly sensitive method for detecting active H. Pylori infection, as it measures the presence of urease, an enzyme produced by the bacteria",
+  "Endoscopy and biopsy, while useful for diagnosing gastric ulcers and other complications of H. Pylori, are more invasive and not the preferred method for detecting residual infection after treatment"
+]</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Urea breath test is more sensitive and non-invasive for detecting H. Pylori</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>7182</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>BRCA-1 postive women have ____% increased risk of breast carcinoma</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F31" t="b">
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>[
+  "Identify the relationship between BRCA-1 and breast cancer risk",
+  "Recognize that BRCA-1 is a high-risk gene mutation for breast cancer",
+  "Recall that BRCA-1 positive women have a significantly increased risk, typically cited as 60-70% by age 80"
+]</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>BRCA-1 positive women have a substantially increased risk of breast carcinoma</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J31" t="b">
+        <v>1</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>[
+  "Identify the known risk associated with BRCA-1 positivity",
+  "Recognize that BRCA-1 positivity significantly increases the risk of breast carcinoma, with most sources indicating a risk substantially higher than the general population",
+  "Compare the provided options to determine which aligns with established medical knowledge, where a 60% increased risk is more plausible for BRCA-1 carriers than a 20% increased risk"
+]</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>BRCA-1 carriers have a substantially increased risk of breast cancer</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="R31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>[
+  "Identify the increased risk of breast carcinoma in BRCA-1 positive women",
+  "Recall that BRCA-1 mutations significantly increase the risk of breast cancer, with most studies indicating a risk between 45% to 72% by age 80",
+  "Compare the provided options to the known risk range"
+]</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>BRCA-1 positive women have a substantially increased risk of breast carcinoma, with a lifetime risk often cited around 60-70%</t>
         </is>
       </c>
     </row>

</xml_diff>